<commit_message>
Ralph iteration 2: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cape Colony" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Northern Cape" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eastern Cape" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="West Transvaal" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eastern Transvaal" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Northern Transvaal" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transorangia" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drakensberg" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Botswana" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lourenço Marques" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zambezi" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hereroland" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Namaqualand" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cape Colony" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Northern Cape" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Eastern Cape" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="West Transvaal" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Eastern Transvaal" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Northern Transvaal" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Transorangia" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Drakensberg" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Botswana" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Lourenço Marques" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Zambezi" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Hereroland" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Namaqualand" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2142,14 +2142,14 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E89" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="90">
@@ -9695,17 +9695,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Historical</t>
+          <t>Unchanged</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>No change</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ralph iteration 3: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cape Colony" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Northern Cape" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Eastern Cape" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="West Transvaal" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Eastern Transvaal" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Northern Transvaal" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Transorangia" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Drakensberg" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Botswana" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Lourenço Marques" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Zambezi" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Hereroland" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Namaqualand" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cape Colony" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Northern Cape" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eastern Cape" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="West Transvaal" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eastern Transvaal" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Northern Transvaal" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transorangia" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drakensberg" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Botswana" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lourenço Marques" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zambezi" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hereroland" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Namaqualand" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -609,10 +609,10 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D11" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12">
@@ -1229,10 +1229,10 @@
         <v>0</v>
       </c>
       <c r="D44" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -1544,10 +1544,10 @@
         <v>0</v>
       </c>
       <c r="D59" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E59" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="60">
@@ -2163,14 +2163,14 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E90" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="91">
@@ -10510,7 +10510,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9">
@@ -10520,7 +10520,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-115</v>
+        <v>-118</v>
       </c>
     </row>
     <row r="10"/>
@@ -11188,15 +11188,15 @@
         <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Historical</t>
+          <t>Exception</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
Ralph iteration 4: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -689,10 +689,10 @@
         <v>36</v>
       </c>
       <c r="C16" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D16" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17">
@@ -1334,10 +1334,10 @@
         <v>12</v>
       </c>
       <c r="D49" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="E49" t="n">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="50">
@@ -1649,10 +1649,10 @@
         <v>36</v>
       </c>
       <c r="D64" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="E64" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="65">
@@ -2184,14 +2184,14 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E91" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="92">
@@ -11518,7 +11518,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9">
@@ -11528,7 +11528,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-81</v>
+        <v>-77</v>
       </c>
     </row>
     <row r="10"/>
@@ -12326,7 +12326,7 @@
         <v>12</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -12334,7 +12334,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>-12</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="39">

</xml_diff>

<commit_message>
Ralph iteration 5: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -2205,14 +2205,14 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E92" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="93">
@@ -12464,7 +12464,7 @@
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -13104,7 +13104,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Historical</t>
+          <t>Counterfactual</t>
         </is>
       </c>
       <c r="F29" t="n">

</xml_diff>

<commit_message>
Ralph iteration 6: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -2226,14 +2226,14 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E93" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="94">

</xml_diff>

<commit_message>
Ralph iteration 7: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -2247,14 +2247,14 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E94" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="95">

</xml_diff>

<commit_message>
Ralph iteration 8: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -689,10 +689,10 @@
         <v>36</v>
       </c>
       <c r="C16" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D16" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17">
@@ -2268,14 +2268,14 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E95" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="96">
@@ -2446,7 +2446,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -2456,7 +2456,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-88</v>
+        <v>-87</v>
       </c>
     </row>
     <row r="10"/>
@@ -3254,7 +3254,7 @@
         <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">

</xml_diff>

<commit_message>
Ralph iteration 9: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -2289,14 +2289,14 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E96" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="97">

</xml_diff>

<commit_message>
Ralph iteration 1: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cape Colony" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Northern Cape" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eastern Cape" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="West Transvaal" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eastern Transvaal" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Northern Transvaal" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transorangia" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drakensberg" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Botswana" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lourenço Marques" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zambezi" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hereroland" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Namaqualand" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cape Colony" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Northern Cape" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Eastern Cape" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="West Transvaal" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Eastern Transvaal" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Northern Transvaal" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Transorangia" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Drakensberg" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Botswana" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Lourenço Marques" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Zambezi" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Hereroland" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Namaqualand" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2180,14 +2180,14 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E95" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="96">

</xml_diff>

<commit_message>
Ralph iteration 10: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -2369,14 +2369,14 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>accepted</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E104" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="105">

</xml_diff>

<commit_message>
Ralph iteration 11: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -1985,14 +1985,14 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t xml:space="preserve">not started</t>
+          <t xml:space="preserve">accepted</t>
         </is>
       </c>
       <c r="D105">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E105">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="106">

</xml_diff>

<commit_message>
Ralph iteration 12: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -222,10 +222,10 @@
         <v>472</v>
       </c>
       <c r="C15">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D15">
-        <v>-346</v>
+        <v>-348</v>
       </c>
     </row>
     <row r="16">
@@ -302,10 +302,10 @@
         <v>0</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -366,10 +366,10 @@
         <v>36</v>
       </c>
       <c r="C24">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D24">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25">
@@ -2006,14 +2006,14 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t xml:space="preserve">not started</t>
+          <t xml:space="preserve">accepted</t>
         </is>
       </c>
       <c r="D106">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E106">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="107">
@@ -5743,15 +5743,15 @@
         <v>44</v>
       </c>
       <c r="D30">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Counterfactual</t>
         </is>
       </c>
       <c r="F30">
-        <v>-40</v>
+        <v>-42</v>
       </c>
     </row>
     <row r="31">
@@ -5851,7 +5851,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Counterfactual</t>
         </is>
       </c>
       <c r="F34">
@@ -5873,15 +5873,15 @@
         <v>0</v>
       </c>
       <c r="D35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exception</t>
+          <t xml:space="preserve">Counterfactual</t>
         </is>
       </c>
       <c r="F35">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -5977,7 +5977,7 @@
         <v>0</v>
       </c>
       <c r="D39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -5985,7 +5985,7 @@
         </is>
       </c>
       <c r="F39">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">

</xml_diff>

<commit_message>
Ralph iteration 13: work in progress
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -2027,14 +2027,14 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t xml:space="preserve">not started</t>
+          <t xml:space="preserve">accepted</t>
         </is>
       </c>
       <c r="D107">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E107">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="108">
@@ -6111,7 +6111,7 @@
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6782,7 +6782,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Counterfactual</t>
         </is>
       </c>
       <c r="F31">

</xml_diff>

<commit_message>
Finalize resource audit package
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -222,10 +222,10 @@
         <v>472</v>
       </c>
       <c r="C15">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D15">
-        <v>-348</v>
+        <v>-346</v>
       </c>
     </row>
     <row r="16">
@@ -238,10 +238,10 @@
         <v>45</v>
       </c>
       <c r="C16">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D16">
-        <v>-13</v>
+        <v>-14</v>
       </c>
     </row>
     <row r="17">
@@ -270,10 +270,10 @@
         <v>123</v>
       </c>
       <c r="C18">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D18">
-        <v>-90</v>
+        <v>-87</v>
       </c>
     </row>
     <row r="19">
@@ -286,10 +286,10 @@
         <v>0</v>
       </c>
       <c r="C19">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D19">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20">
@@ -334,10 +334,10 @@
         <v>71</v>
       </c>
       <c r="C22">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D22">
-        <v>-40</v>
+        <v>-36</v>
       </c>
     </row>
     <row r="23">
@@ -1199,10 +1199,10 @@
         <v>123</v>
       </c>
       <c r="D66">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E66">
-        <v>-91</v>
+        <v>-90</v>
       </c>
     </row>
     <row r="67">
@@ -1535,10 +1535,10 @@
         <v>0</v>
       </c>
       <c r="D82">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E82">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="83">
@@ -1598,10 +1598,10 @@
         <v>6</v>
       </c>
       <c r="D85">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E85">
-        <v>-6</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="86">
@@ -2048,14 +2048,14 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t xml:space="preserve">not started</t>
+          <t xml:space="preserve">accepted</t>
         </is>
       </c>
       <c r="D108">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E108">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -2153,7 +2153,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>-117</v>
+        <v>-116</v>
       </c>
     </row>
     <row r="12">
@@ -2716,7 +2716,7 @@
         <v>72</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2724,7 +2724,7 @@
         </is>
       </c>
       <c r="F30">
-        <v>-72</v>
+        <v>-71</v>
       </c>
     </row>
     <row r="31">
@@ -2742,15 +2742,15 @@
         <v>5</v>
       </c>
       <c r="D31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Exception</t>
         </is>
       </c>
       <c r="F31">
-        <v>-4</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="32">
@@ -2898,7 +2898,7 @@
         <v>11</v>
       </c>
       <c r="D37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -2906,7 +2906,7 @@
         </is>
       </c>
       <c r="F37">
-        <v>-11</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="38">
@@ -3152,7 +3152,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -3162,7 +3162,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>-86</v>
+        <v>-83</v>
       </c>
     </row>
     <row r="12">
@@ -3725,15 +3725,15 @@
         <v>48</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exception</t>
+          <t xml:space="preserve">Historical</t>
         </is>
       </c>
       <c r="F30">
-        <v>-48</v>
+        <v>-47</v>
       </c>
     </row>
     <row r="31">
@@ -3803,7 +3803,7 @@
         <v>0</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -3811,7 +3811,7 @@
         </is>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -3907,7 +3907,7 @@
         <v>5</v>
       </c>
       <c r="D37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="F37">
-        <v>-5</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="38">
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
@@ -4171,7 +4171,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>-104</v>
+        <v>-103</v>
       </c>
     </row>
     <row r="12">
@@ -4481,7 +4481,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Removed</t>
+          <t xml:space="preserve">No change</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4916,7 @@
         <v>9</v>
       </c>
       <c r="D37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -4924,7 +4924,7 @@
         </is>
       </c>
       <c r="F37">
-        <v>-9</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="38">
@@ -5170,7 +5170,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10">
@@ -5180,7 +5180,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>-89</v>
+        <v>-88</v>
       </c>
     </row>
     <row r="12">
@@ -5821,15 +5821,15 @@
         <v>0</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exception</t>
+          <t xml:space="preserve">Historical</t>
         </is>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -6179,7 +6179,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -6189,7 +6189,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>-69</v>
+        <v>-68</v>
       </c>
     </row>
     <row r="12">
@@ -6934,7 +6934,7 @@
         <v>2</v>
       </c>
       <c r="D37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6942,7 +6942,7 @@
         </is>
       </c>
       <c r="F37">
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="38">
@@ -7188,7 +7188,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -7198,7 +7198,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>-68</v>
+        <v>-67</v>
       </c>
     </row>
     <row r="12">
@@ -7865,15 +7865,15 @@
         <v>0</v>
       </c>
       <c r="D34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exception</t>
+          <t xml:space="preserve">Historical</t>
         </is>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -14251,7 +14251,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10">
@@ -14261,7 +14261,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>-115</v>
+        <v>-114</v>
       </c>
     </row>
     <row r="12">
@@ -14902,7 +14902,7 @@
         <v>30</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -14910,7 +14910,7 @@
         </is>
       </c>
       <c r="F33">
-        <v>-30</v>
+        <v>-29</v>
       </c>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
Release 0.10 Southern Africa patch
</commit_message>
<xml_diff>
--- a/Docs/resources/RESOURCES.xlsx
+++ b/Docs/resources/RESOURCES.xlsx
@@ -2239,17 +2239,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Unchanged</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Added</t>
+          <t xml:space="preserve">No change</t>
         </is>
       </c>
     </row>
@@ -2399,17 +2399,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unchanged</t>
+          <t xml:space="preserve">Historical</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">No change</t>
+          <t xml:space="preserve">Removed</t>
         </is>
       </c>
     </row>
@@ -3376,17 +3376,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Unchanged</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Added</t>
+          <t xml:space="preserve">No change</t>
         </is>
       </c>
     </row>
@@ -4417,17 +4417,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unchanged</t>
+          <t xml:space="preserve">Historical</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">No change</t>
+          <t xml:space="preserve">Removed</t>
         </is>
       </c>
     </row>
@@ -4481,7 +4481,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">No change</t>
+          <t xml:space="preserve">Removed</t>
         </is>
       </c>
     </row>
@@ -4609,17 +4609,17 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Unchanged</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Added</t>
+          <t xml:space="preserve">No change</t>
         </is>
       </c>
     </row>
@@ -5266,17 +5266,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Unchanged</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Added</t>
+          <t xml:space="preserve">No change</t>
         </is>
       </c>
     </row>
@@ -5426,17 +5426,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unchanged</t>
+          <t xml:space="preserve">Historical</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">No change</t>
+          <t xml:space="preserve">Removed</t>
         </is>
       </c>
     </row>
@@ -6275,17 +6275,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Unchanged</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Added</t>
+          <t xml:space="preserve">No change</t>
         </is>
       </c>
     </row>
@@ -6403,17 +6403,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Unchanged</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Added</t>
+          <t xml:space="preserve">No change</t>
         </is>
       </c>
     </row>
@@ -9430,17 +9430,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Unchanged</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Added</t>
+          <t xml:space="preserve">No change</t>
         </is>
       </c>
     </row>
@@ -9462,17 +9462,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Unchanged</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Added</t>
+          <t xml:space="preserve">No change</t>
         </is>
       </c>
     </row>
@@ -10147,7 +10147,7 @@
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
   </cols>
   <sheetData>
@@ -10311,17 +10311,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unchanged</t>
+          <t xml:space="preserve">Historical</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">No change</t>
+          <t xml:space="preserve">Removed</t>
         </is>
       </c>
     </row>
@@ -10407,17 +10407,17 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Counterfactual</t>
+          <t xml:space="preserve">Historical</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">No change</t>
+          <t xml:space="preserve">Removed</t>
         </is>
       </c>
     </row>
@@ -11480,17 +11480,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unchanged</t>
+          <t xml:space="preserve">Historical</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">No change</t>
+          <t xml:space="preserve">Removed</t>
         </is>
       </c>
     </row>
@@ -14347,17 +14347,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historical</t>
+          <t xml:space="preserve">Unchanged</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Added</t>
+          <t xml:space="preserve">No change</t>
         </is>
       </c>
     </row>
@@ -15516,17 +15516,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unchanged</t>
+          <t xml:space="preserve">Historical</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">No change</t>
+          <t xml:space="preserve">Removed</t>
         </is>
       </c>
     </row>

</xml_diff>